<commit_message>
feat: update test fixture verification to include quantidadeServidores validation
</commit_message>
<xml_diff>
--- a/tests/fixtures/test-lancamentos.xlsx
+++ b/tests/fixtures/test-lancamentos.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H6"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -406,6 +406,7 @@
     <col min="5" max="5" width="10.83203125" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" customWidth="1"/>
     <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -430,6 +431,9 @@
       <c r="G1" t="str">
         <v>FolhaSuplementar</v>
       </c>
+      <c r="H1" t="str">
+        <v>quantidadeServidores</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -453,6 +457,9 @@
       <c r="G2">
         <v>0</v>
       </c>
+      <c r="H2">
+        <v>5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -476,6 +483,9 @@
       <c r="G3">
         <v>0</v>
       </c>
+      <c r="H3">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -499,6 +509,9 @@
       <c r="G4">
         <v>5000</v>
       </c>
+      <c r="H4">
+        <v>8</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -522,6 +535,9 @@
       <c r="G5">
         <v>0</v>
       </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -545,10 +561,13 @@
       <c r="G6">
         <v>3000</v>
       </c>
+      <c r="H6">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>